<commit_message>
Azure blob, sharepoint update and PW upload update
</commit_message>
<xml_diff>
--- a/MPDT_FileGeneration_ModelNumberPatch/Input/Planting MPDT Asset Matchup1.xlsx
+++ b/MPDT_FileGeneration_ModelNumberPatch/Input/Planting MPDT Asset Matchup1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://arcadiso365-my.sharepoint.com/personal/nirmala_seethappan_arcadis_com/Documents/Documents/GitHub/MPDT_FileGeneration_ModelNumberPatch/Input/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nxic2385\Documents\GitHub\Arc_Datapipelines\MPDT_FileGeneration_ModelNumberPatch\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="54" documentId="8_{A1D6F51A-260D-4B77-9B7D-7E1778CE0F8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{38BDB39F-9303-4544-A546-983EBDF3221E}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{840EFA39-AB94-4162-A61A-DF1EEF6C1310}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{931FFE6B-42CC-4CAD-9839-EDDB28A0ADD1}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{931FFE6B-42CC-4CAD-9839-EDDB28A0ADD1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -41,12 +41,15 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24063" uniqueCount="2786">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24057" uniqueCount="2788">
   <si>
     <t>Level 2 UAID</t>
   </si>
@@ -8404,6 +8407,12 @@
   </si>
   <si>
     <t>1MC06-CEK-CV-FRM-CS03_CL05-000069</t>
+  </si>
+  <si>
+    <t>HS2-00003B936</t>
+  </si>
+  <si>
+    <t>Calvert Cutting Planting Plot 2</t>
   </si>
 </sst>
 </file>
@@ -8447,13 +8456,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -8793,7 +8803,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4714BB8D-9A6F-47D4-9BEE-35719620A990}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15.81640625" bestFit="1" customWidth="1"/>
@@ -8817,36 +8827,14 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>2777</v>
-      </c>
-      <c r="B2" t="s">
-        <v>2780</v>
-      </c>
-      <c r="C2" t="s">
-        <v>2781</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>2778</v>
-      </c>
-      <c r="B3" t="s">
-        <v>2782</v>
-      </c>
-      <c r="C3" t="s">
-        <v>2783</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>2779</v>
-      </c>
-      <c r="B4" t="s">
-        <v>2784</v>
-      </c>
-      <c r="C4" t="s">
-        <v>2785</v>
+      <c r="A2" s="4" t="s">
+        <v>2786</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>2787</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>2655</v>
       </c>
     </row>
   </sheetData>

</xml_diff>